<commit_message>
Fix platform-owner check broken by skylinx->emplinx owner rename
is_platform_owner was hardcoded to username=="skylinx" (base/rbac.py) and
re-checked in base/middleware._is_platform_owner. After the owner account was
renamed to "emplinx", the real owner was NO LONGER recognized as platform
owner -> lost the "All companies" switcher and got hard-locked to a single
tenant like a regular user; manager scoping also treated them as a scoped user.

Define platform owner as is_superuser (tenants are always non-superuser Company
Admins, so superuser is the operator marker) — survives any username rename.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/worklog.xlsx
+++ b/docs/worklog.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F344"/>
+  <dimension ref="A1:F360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11447,6 +11447,518 @@
         </is>
       </c>
     </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>01:24</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E345" s="2" t="inlineStr">
+        <is>
+          <t>Smoke-test round 2: remaining export + notification-sound crashes</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>dfb86e27</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>01:21</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E346" s="2" t="inlineStr">
+        <is>
+          <t>Smoke-test audit: fix 9 crashing endpoints across modules</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>98570f2e</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>00:52</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E347" s="2" t="inlineStr">
+        <is>
+          <t>Fix Python 3.8 import crash in announcement API (list[dict] hint)</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>54d174ac</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>Offboarding audit: resignation-delete IDOR, unguarded gets, UTC notice date</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>45964406</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>00:40</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E349" s="2" t="inlineStr">
+        <is>
+          <t>Project audit: fix undefined-date 500, cross-project stage move, employee_get crash</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>dcd04456</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>00:27</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E350" s="2" t="inlineStr">
+        <is>
+          <t>Asset audit: fix list-view crash, asset-count 500, dead duplicate manager</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>3b064d68</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>00:21</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E351" s="2" t="inlineStr">
+        <is>
+          <t>PMS audit: feedback submit IDOR, objective-view crash, feedback close-loop bug</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>82ac3bbf</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>00:13</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>Recruitment audit: survey perm gap, 2 crashes, delete-order data loss, UTC</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>e17cfeb5</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>evening</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Geofencing</t>
+        </is>
+      </c>
+      <c r="E353" s="2" t="inlineStr">
+        <is>
+          <t>Added GeoFencing.enforce BooleanField (default False, opt-in) so out-of-zone check-in/out can be hard-blocked instead of just flagged + admin-notified</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>geofencing/models.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>evening</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Attendance/Mobile</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>MobileCheckInAPIView and MobileCheckOutAPIView now return 400 OUTSIDE_GEOFENCE (with distanceFromCenterMeters) when within_geofence is False and geofence.enforce is True</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>skylinx_api/api_views/attendance/mobile_views.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>evening</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Attendance</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>Removed stray `from datetime import timezone` in views.py that was shadowing django.utils.timezone and silently breaking .now()/.localtime() calls in this file</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>skylinx_api/api_views/attendance/views.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>evening</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Attendance</t>
+        </is>
+      </c>
+      <c r="E356" s="2" t="inlineStr">
+        <is>
+          <t>ClockInAPIView day-row lookup (today + yesterday) no longer raises DoesNotExist when EmployeeShiftDay's company M2M is unlinked for the tenant: falls back through company-scoped filter -&gt; entire() -&gt; create(day=...)</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>skylinx_api/api_views/attendance/views.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>23:56</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>Employee audit: fix document IDOR, anon dynamic-create, 2 crashes, UTC dates</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>89227295</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>22:58</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>Leave audit: fix bulk-delete IDOR + 3 unguarded .get() 500s</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>09c0ed9c</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="inlineStr">
+        <is>
+          <t>Payroll audit: fix perm gap, null-wage/rate crashes, UTC month bugs</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>cbf40aa8</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>21:13</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="E360" s="2" t="inlineStr">
+        <is>
+          <t>Audit attendance: fix API crashes, add configurable geofence enforcement</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>a65effb3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>